<commit_message>
Completed Week 4 air quality inference exercise
</commit_message>
<xml_diff>
--- a/final_project/11-14-25 SM Competition Data Template.xlsx
+++ b/final_project/11-14-25 SM Competition Data Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mallo/Documents/Projects/biol696/collins_mallory_biol696_workflows/final_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1B5E735-0EC1-3444-B8BC-36878ADBFF47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC1064C-05B7-9F48-B0A9-53DC5E383B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16100" activeTab="1" xr2:uid="{F461D164-D39E-5F43-8C81-7877C5AB1617}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16100" xr2:uid="{F461D164-D39E-5F43-8C81-7877C5AB1617}"/>
   </bookViews>
   <sheets>
     <sheet name="CFU" sheetId="1" r:id="rId1"/>

</xml_diff>